<commit_message>
making changes to detecting missed last checkpoint cut off and retired. Example POLISH fella/ Gressoney -> Gressoney IN instead of just Gressoney. THis caused serious issues when looking at missed cut offs and very inaccurate picture.
</commit_message>
<xml_diff>
--- a/TOR330 Data/4. TOR330 Timetable Data/TOR330_aid_station_cut_offs_df.xlsx
+++ b/TOR330 Data/4. TOR330 Timetable Data/TOR330_aid_station_cut_offs_df.xlsx
@@ -1,20 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karina\Portfolio\TORX\TOR330 Data\4. TOR330 Timetable Data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3256A2C1-EE4C-4E14-8F10-6F5146C3ED6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="71">
   <si>
     <t>Aid Station</t>
   </si>
@@ -227,13 +246,16 @@
   </si>
   <si>
     <t>Stage 7</t>
+  </si>
+  <si>
+    <t>Oyace IN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,13 +318,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -340,7 +370,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -374,6 +404,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -408,9 +439,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -583,11 +615,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I49"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -616,7 +648,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -636,7 +668,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -665,7 +697,7 @@
         <v>19800</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -685,7 +717,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -705,7 +737,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -734,7 +766,7 @@
         <v>68400</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -763,7 +795,7 @@
         <v>75600</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -774,7 +806,7 @@
         <v>5176</v>
       </c>
       <c r="D8">
-        <v>6.340000000000003</v>
+        <v>6.3400000000000034</v>
       </c>
       <c r="E8">
         <v>837</v>
@@ -783,7 +815,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -794,7 +826,7 @@
         <v>5750</v>
       </c>
       <c r="D9">
-        <v>7.969999999999999</v>
+        <v>7.9699999999999989</v>
       </c>
       <c r="E9">
         <v>574</v>
@@ -803,18 +835,18 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
       <c r="B10">
-        <v>78.26000000000001</v>
+        <v>78.260000000000005</v>
       </c>
       <c r="C10">
         <v>7174</v>
       </c>
       <c r="D10">
-        <v>15.40000000000001</v>
+        <v>15.400000000000009</v>
       </c>
       <c r="E10">
         <v>1424</v>
@@ -832,7 +864,7 @@
         <v>120600</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -843,7 +875,7 @@
         <v>9126</v>
       </c>
       <c r="D11">
-        <v>16.89999999999999</v>
+        <v>16.899999999999991</v>
       </c>
       <c r="E11">
         <v>1952</v>
@@ -852,7 +884,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -863,7 +895,7 @@
         <v>9282</v>
       </c>
       <c r="D12">
-        <v>8.840000000000003</v>
+        <v>8.8400000000000034</v>
       </c>
       <c r="E12">
         <v>156</v>
@@ -881,7 +913,7 @@
         <v>151200</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -910,7 +942,7 @@
         <v>158400</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -921,7 +953,7 @@
         <v>9801</v>
       </c>
       <c r="D14">
-        <v>5.780000000000001</v>
+        <v>5.7800000000000011</v>
       </c>
       <c r="E14">
         <v>519</v>
@@ -930,7 +962,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -941,7 +973,7 @@
         <v>11020</v>
       </c>
       <c r="D15">
-        <v>16.17</v>
+        <v>16.170000000000002</v>
       </c>
       <c r="E15">
         <v>1219</v>
@@ -950,18 +982,18 @@
         <v>61</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
       <c r="B16">
-        <v>131.45</v>
+        <v>131.44999999999999</v>
       </c>
       <c r="C16">
         <v>11110</v>
       </c>
       <c r="D16">
-        <v>5.499999999999986</v>
+        <v>5.4999999999999858</v>
       </c>
       <c r="E16">
         <v>90</v>
@@ -970,12 +1002,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>24</v>
       </c>
       <c r="B17">
-        <v>139.36</v>
+        <v>139.36000000000001</v>
       </c>
       <c r="C17">
         <v>11353</v>
@@ -990,12 +1022,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>25</v>
       </c>
       <c r="B18">
-        <v>149.77</v>
+        <v>149.77000000000001</v>
       </c>
       <c r="C18">
         <v>12050</v>
@@ -1010,7 +1042,7 @@
         <v>25</v>
       </c>
       <c r="G18">
-        <v>64800.00000000001</v>
+        <v>64800.000000000007</v>
       </c>
       <c r="H18" t="s">
         <v>61</v>
@@ -1019,12 +1051,12 @@
         <v>223200</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>26</v>
       </c>
       <c r="B19">
-        <v>149.77</v>
+        <v>149.77000000000001</v>
       </c>
       <c r="C19">
         <v>12050</v>
@@ -1048,7 +1080,7 @@
         <v>230400</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -1068,7 +1100,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1079,7 +1111,7 @@
         <v>13935</v>
       </c>
       <c r="D21">
-        <v>7.310000000000002</v>
+        <v>7.3100000000000023</v>
       </c>
       <c r="E21">
         <v>1240</v>
@@ -1088,7 +1120,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -1099,7 +1131,7 @@
         <v>14814</v>
       </c>
       <c r="D22">
-        <v>4.439999999999998</v>
+        <v>4.4399999999999977</v>
       </c>
       <c r="E22">
         <v>879</v>
@@ -1108,7 +1140,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -1119,7 +1151,7 @@
         <v>15512</v>
       </c>
       <c r="D23">
-        <v>8.47999999999999</v>
+        <v>8.4799999999999898</v>
       </c>
       <c r="E23">
         <v>698</v>
@@ -1137,7 +1169,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>31</v>
       </c>
@@ -1148,7 +1180,7 @@
         <v>16049</v>
       </c>
       <c r="D24">
-        <v>5.300000000000011</v>
+        <v>5.3000000000000114</v>
       </c>
       <c r="E24">
         <v>537</v>
@@ -1157,7 +1189,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -1177,7 +1209,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -1188,7 +1220,7 @@
         <v>16989</v>
       </c>
       <c r="D26">
-        <v>5.590000000000003</v>
+        <v>5.5900000000000034</v>
       </c>
       <c r="E26">
         <v>375</v>
@@ -1206,7 +1238,7 @@
         <v>293400</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -1217,7 +1249,7 @@
         <v>17856</v>
       </c>
       <c r="D27">
-        <v>6.20999999999998</v>
+        <v>6.2099999999999804</v>
       </c>
       <c r="E27">
         <v>867</v>
@@ -1226,7 +1258,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>35</v>
       </c>
@@ -1237,7 +1269,7 @@
         <v>17983</v>
       </c>
       <c r="D28">
-        <v>7.110000000000014</v>
+        <v>7.1100000000000136</v>
       </c>
       <c r="E28">
         <v>127</v>
@@ -1255,7 +1287,7 @@
         <v>306000</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -1284,7 +1316,7 @@
         <v>313200</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -1295,7 +1327,7 @@
         <v>18515</v>
       </c>
       <c r="D30">
-        <v>5.080000000000013</v>
+        <v>5.0800000000000134</v>
       </c>
       <c r="E30">
         <v>532</v>
@@ -1304,7 +1336,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -1315,7 +1347,7 @@
         <v>19674</v>
       </c>
       <c r="D31">
-        <v>11.89999999999998</v>
+        <v>11.899999999999981</v>
       </c>
       <c r="E31">
         <v>1159</v>
@@ -1333,7 +1365,7 @@
         <v>356400</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>39</v>
       </c>
@@ -1344,7 +1376,7 @@
         <v>20722</v>
       </c>
       <c r="D32">
-        <v>7.800000000000011</v>
+        <v>7.8000000000000114</v>
       </c>
       <c r="E32">
         <v>1048</v>
@@ -1353,7 +1385,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -1364,7 +1396,7 @@
         <v>21077</v>
       </c>
       <c r="D33">
-        <v>8.840000000000003</v>
+        <v>8.8400000000000034</v>
       </c>
       <c r="E33">
         <v>355</v>
@@ -1382,7 +1414,7 @@
         <v>378000</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>41</v>
       </c>
@@ -1411,7 +1443,7 @@
         <v>385200</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -1422,7 +1454,7 @@
         <v>21912</v>
       </c>
       <c r="D35">
-        <v>4.879999999999995</v>
+        <v>4.8799999999999946</v>
       </c>
       <c r="E35">
         <v>835</v>
@@ -1431,7 +1463,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>43</v>
       </c>
@@ -1442,7 +1474,7 @@
         <v>22323</v>
       </c>
       <c r="D36">
-        <v>5.009999999999991</v>
+        <v>5.0099999999999909</v>
       </c>
       <c r="E36">
         <v>411</v>
@@ -1451,7 +1483,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>44</v>
       </c>
@@ -1462,7 +1494,7 @@
         <v>22956</v>
       </c>
       <c r="D37">
-        <v>8.450000000000017</v>
+        <v>8.4500000000000171</v>
       </c>
       <c r="E37">
         <v>633</v>
@@ -1471,18 +1503,18 @@
         <v>67</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>45</v>
       </c>
       <c r="B38">
-        <v>259.41</v>
+        <v>259.41000000000003</v>
       </c>
       <c r="C38">
         <v>23639</v>
       </c>
       <c r="D38">
-        <v>3.450000000000017</v>
+        <v>3.4500000000000171</v>
       </c>
       <c r="E38">
         <v>683</v>
@@ -1491,7 +1523,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>46</v>
       </c>
@@ -1511,230 +1543,254 @@
         <v>67</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="B40">
-        <v>277.83</v>
+        <v>273.8</v>
       </c>
       <c r="C40">
-        <v>25178</v>
+        <v>24283</v>
       </c>
       <c r="D40">
-        <v>13.82999999999998</v>
+        <f>(B40-B39)</f>
+        <v>9.8000000000000114</v>
       </c>
       <c r="E40">
-        <v>1149</v>
+        <f>(C40-C39)</f>
+        <v>254</v>
       </c>
       <c r="H40" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B41">
-        <v>285.66</v>
+        <v>277.83</v>
       </c>
       <c r="C41">
-        <v>25702</v>
+        <v>25178</v>
       </c>
       <c r="D41">
-        <v>7.830000000000041</v>
+        <f>(B41-B40)</f>
+        <v>4.0299999999999727</v>
       </c>
       <c r="E41">
-        <v>524</v>
-      </c>
-      <c r="F41" t="s">
-        <v>48</v>
-      </c>
-      <c r="G41">
-        <v>18000</v>
+        <f>(C41-C40)</f>
+        <v>895</v>
       </c>
       <c r="H41" t="s">
         <v>67</v>
       </c>
-      <c r="I41">
-        <v>403200</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9">
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B42">
-        <v>285.66</v>
+        <v>285.66000000000003</v>
       </c>
       <c r="C42">
         <v>25702</v>
       </c>
       <c r="D42">
+        <v>7.8300000000000409</v>
+      </c>
+      <c r="E42">
+        <v>524</v>
+      </c>
+      <c r="F42" t="s">
+        <v>48</v>
+      </c>
+      <c r="G42">
+        <v>18000</v>
+      </c>
+      <c r="H42" t="s">
+        <v>67</v>
+      </c>
+      <c r="I42">
+        <v>403200</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43">
+        <v>285.66000000000003</v>
+      </c>
+      <c r="C43">
+        <v>25702</v>
+      </c>
+      <c r="D43">
         <v>0</v>
       </c>
-      <c r="E42">
+      <c r="E43">
         <v>0</v>
       </c>
-      <c r="F42" t="s">
+      <c r="F43" t="s">
         <v>49</v>
       </c>
-      <c r="G42">
+      <c r="G43">
         <v>7200</v>
       </c>
-      <c r="H42" t="s">
+      <c r="H43" t="s">
         <v>68</v>
       </c>
-      <c r="I42">
+      <c r="I43">
         <v>410400</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
-      <c r="A43" t="s">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>50</v>
       </c>
-      <c r="B43">
+      <c r="B44">
         <v>290.3</v>
       </c>
-      <c r="C43">
+      <c r="C44">
         <v>26763</v>
       </c>
-      <c r="D43">
-        <v>4.639999999999986</v>
-      </c>
-      <c r="E43">
+      <c r="D44">
+        <v>4.6399999999999864</v>
+      </c>
+      <c r="E44">
         <v>1061</v>
-      </c>
-      <c r="H43" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9">
-      <c r="A44" t="s">
-        <v>51</v>
-      </c>
-      <c r="B44">
-        <v>296.86</v>
-      </c>
-      <c r="C44">
-        <v>27181</v>
-      </c>
-      <c r="D44">
-        <v>6.560000000000002</v>
-      </c>
-      <c r="E44">
-        <v>418</v>
       </c>
       <c r="H44" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B45">
-        <v>306.98</v>
+        <v>296.86</v>
       </c>
       <c r="C45">
-        <v>27503</v>
+        <v>27181</v>
       </c>
       <c r="D45">
-        <v>10.12</v>
+        <v>6.5600000000000023</v>
       </c>
       <c r="E45">
-        <v>322</v>
+        <v>418</v>
       </c>
       <c r="H45" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B46">
-        <v>316.09</v>
+        <v>306.98</v>
       </c>
       <c r="C46">
-        <v>28667</v>
+        <v>27503</v>
       </c>
       <c r="D46">
-        <v>9.109999999999957</v>
+        <v>10.119999999999999</v>
       </c>
       <c r="E46">
-        <v>1164</v>
+        <v>322</v>
       </c>
       <c r="H46" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B47">
-        <v>321.93</v>
+        <v>316.08999999999997</v>
       </c>
       <c r="C47">
-        <v>29257</v>
+        <v>28667</v>
       </c>
       <c r="D47">
-        <v>5.840000000000032</v>
+        <v>9.1099999999999568</v>
       </c>
       <c r="E47">
-        <v>590</v>
+        <v>1164</v>
       </c>
       <c r="H47" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B48">
-        <v>330.71</v>
+        <v>321.93</v>
       </c>
       <c r="C48">
-        <v>29567</v>
+        <v>29257</v>
       </c>
       <c r="D48">
-        <v>8.779999999999973</v>
+        <v>5.8400000000000318</v>
       </c>
       <c r="E48">
-        <v>310</v>
+        <v>590</v>
       </c>
       <c r="H48" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B49">
-        <v>335.32</v>
+        <v>330.71</v>
       </c>
       <c r="C49">
-        <v>29608</v>
+        <v>29567</v>
       </c>
       <c r="D49">
-        <v>4.610000000000014</v>
+        <v>8.7799999999999727</v>
       </c>
       <c r="E49">
-        <v>41</v>
-      </c>
-      <c r="F49" t="s">
-        <v>56</v>
-      </c>
-      <c r="G49">
-        <v>75600</v>
+        <v>310</v>
       </c>
       <c r="H49" t="s">
         <v>69</v>
       </c>
-      <c r="I49">
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50">
+        <v>335.32</v>
+      </c>
+      <c r="C50">
+        <v>29608</v>
+      </c>
+      <c r="D50">
+        <v>4.6100000000000136</v>
+      </c>
+      <c r="E50">
+        <v>41</v>
+      </c>
+      <c r="F50" t="s">
+        <v>56</v>
+      </c>
+      <c r="G50">
+        <v>75600</v>
+      </c>
+      <c r="H50" t="s">
+        <v>69</v>
+      </c>
+      <c r="I50">
         <v>486000</v>
       </c>
     </row>

</xml_diff>